<commit_message>
Republish Tacen_2025_WC: Kayak Cross individual (Time Trials) RANK from official classification (97 cells; maintainer 2026-10-21)
</commit_message>
<xml_diff>
--- a/events/Tacen_2025_WC/Tacen_2025_WC_start.xlsx
+++ b/events/Tacen_2025_WC/Tacen_2025_WC_start.xlsx
@@ -15671,6 +15671,11 @@
       <c r="K254" t="n">
         <v>253</v>
       </c>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="R254" t="inlineStr">
         <is>
           <t>LUKNAROVA Emanuela</t>
@@ -15734,6 +15739,11 @@
       <c r="K255" t="n">
         <v>254</v>
       </c>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="R255" t="inlineStr">
         <is>
           <t>NAGASU Momoka</t>
@@ -15797,6 +15807,11 @@
       <c r="K256" t="n">
         <v>255</v>
       </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="R256" t="inlineStr">
         <is>
           <t>PITCHER FARRELL Cleo</t>
@@ -15860,6 +15875,11 @@
       <c r="K257" t="n">
         <v>256</v>
       </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="R257" t="inlineStr">
         <is>
           <t>DUC Jessica</t>
@@ -15986,6 +16006,11 @@
       <c r="K259" t="n">
         <v>258</v>
       </c>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="R259" t="inlineStr">
         <is>
           <t>CROSBEE Sarah</t>
@@ -16049,6 +16074,11 @@
       <c r="K260" t="n">
         <v>259</v>
       </c>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="R260" t="inlineStr">
         <is>
           <t>MATTI Svenja</t>
@@ -16112,6 +16142,11 @@
       <c r="K261" t="n">
         <v>260</v>
       </c>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="R261" t="inlineStr">
         <is>
           <t>REX Rosie</t>
@@ -16175,6 +16210,11 @@
       <c r="K262" t="n">
         <v>261</v>
       </c>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="R262" t="inlineStr">
         <is>
           <t>SRIBAR Ria</t>
@@ -16238,6 +16278,11 @@
       <c r="K263" t="n">
         <v>262</v>
       </c>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="R263" t="inlineStr">
         <is>
           <t>GORA Aleksandra</t>
@@ -16301,6 +16346,11 @@
       <c r="K264" t="n">
         <v>263</v>
       </c>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="R264" t="inlineStr">
         <is>
           <t>BRZESKA Dominika</t>
@@ -16364,6 +16414,11 @@
       <c r="K265" t="n">
         <v>264</v>
       </c>
+      <c r="M265" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="R265" t="inlineStr">
         <is>
           <t>O'CALLAGHAN Georgia</t>
@@ -16427,6 +16482,11 @@
       <c r="K266" t="n">
         <v>265</v>
       </c>
+      <c r="M266" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="R266" t="inlineStr">
         <is>
           <t>SORRIBES Laia</t>
@@ -16490,6 +16550,11 @@
       <c r="K267" t="n">
         <v>266</v>
       </c>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="R267" t="inlineStr">
         <is>
           <t>HILGERTOVA Amalie</t>
@@ -16553,6 +16618,11 @@
       <c r="K268" t="n">
         <v>267</v>
       </c>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="R268" t="inlineStr">
         <is>
           <t>ALTMAN Marcella</t>
@@ -16616,6 +16686,11 @@
       <c r="K269" t="n">
         <v>268</v>
       </c>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="R269" t="inlineStr">
         <is>
           <t>HERZOG Andrea</t>
@@ -16679,6 +16754,11 @@
       <c r="K270" t="n">
         <v>269</v>
       </c>
+      <c r="M270" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="R270" t="inlineStr">
         <is>
           <t>PANKOVA Zuzana</t>
@@ -16742,6 +16822,11 @@
       <c r="K271" t="n">
         <v>270</v>
       </c>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="R271" t="inlineStr">
         <is>
           <t>SAMKOVA Olga</t>
@@ -16805,6 +16890,11 @@
       <c r="K272" t="n">
         <v>271</v>
       </c>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="R272" t="inlineStr">
         <is>
           <t>STANOVSKA Sona</t>
@@ -16868,6 +16958,11 @@
       <c r="K273" t="n">
         <v>272</v>
       </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="R273" t="inlineStr">
         <is>
           <t>LEAVER Lois</t>
@@ -16931,6 +17026,11 @@
       <c r="K274" t="n">
         <v>273</v>
       </c>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
       <c r="R274" t="inlineStr">
         <is>
           <t>LI Shiting</t>
@@ -16994,6 +17094,11 @@
       <c r="K275" t="n">
         <v>274</v>
       </c>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="R275" t="inlineStr">
         <is>
           <t>BAYN Nele</t>
@@ -17057,6 +17162,11 @@
       <c r="K276" t="n">
         <v>275</v>
       </c>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="R276" t="inlineStr">
         <is>
           <t>PINTERIC Naja</t>
@@ -17120,6 +17230,11 @@
       <c r="K277" t="n">
         <v>276</v>
       </c>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="R277" t="inlineStr">
         <is>
           <t>NOVAK Ajda</t>
@@ -17183,6 +17298,11 @@
       <c r="K278" t="n">
         <v>277</v>
       </c>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="R278" t="inlineStr">
         <is>
           <t>TEUNISSEN Lena</t>
@@ -17246,6 +17366,11 @@
       <c r="K279" t="n">
         <v>278</v>
       </c>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R279" t="inlineStr">
         <is>
           <t>HOCEVAR Eva Alina</t>
@@ -17309,6 +17434,11 @@
       <c r="K280" t="n">
         <v>279</v>
       </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="R280" t="inlineStr">
         <is>
           <t>US Viktoriia</t>
@@ -17372,6 +17502,11 @@
       <c r="K281" t="n">
         <v>280</v>
       </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="R281" t="inlineStr">
         <is>
           <t>SABATTINI Chiara</t>
@@ -17435,6 +17570,11 @@
       <c r="K282" t="n">
         <v>281</v>
       </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="R282" t="inlineStr">
         <is>
           <t>LAZKANO Miren</t>
@@ -17498,6 +17638,11 @@
       <c r="K283" t="n">
         <v>282</v>
       </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="R283" t="inlineStr">
         <is>
           <t>SATILA Ana</t>
@@ -17561,6 +17706,11 @@
       <c r="K284" t="n">
         <v>283</v>
       </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="R284" t="inlineStr">
         <is>
           <t>ZWOLINSKA Klaudia</t>
@@ -17624,6 +17774,11 @@
       <c r="K285" t="n">
         <v>284</v>
       </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="R285" t="inlineStr">
         <is>
           <t>DORIA Monica</t>
@@ -17687,6 +17842,11 @@
       <c r="K286" t="n">
         <v>285</v>
       </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="R286" t="inlineStr">
         <is>
           <t>ESTACIA NETA Omira</t>
@@ -17750,6 +17910,11 @@
       <c r="K287" t="n">
         <v>286</v>
       </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="R287" t="inlineStr">
         <is>
           <t>KNEBLOVA Tereza</t>
@@ -17813,6 +17978,11 @@
       <c r="K288" t="n">
         <v>287</v>
       </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="R288" t="inlineStr">
         <is>
           <t>SETCHELL Nikita</t>
@@ -17876,6 +18046,11 @@
       <c r="K289" t="n">
         <v>288</v>
       </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="R289" t="inlineStr">
         <is>
           <t>VUITTON Emma</t>
@@ -17939,6 +18114,11 @@
       <c r="K290" t="n">
         <v>289</v>
       </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="R290" t="inlineStr">
         <is>
           <t>LEIBFARTH Evy</t>
@@ -18002,6 +18182,11 @@
       <c r="K291" t="n">
         <v>290</v>
       </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="R291" t="inlineStr">
         <is>
           <t>FUNK Ricarda</t>
@@ -18065,6 +18250,11 @@
       <c r="K292" t="n">
         <v>291</v>
       </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
       <c r="R292" t="inlineStr">
         <is>
           <t>CHOURRAUT Maialen</t>
@@ -18128,6 +18318,11 @@
       <c r="K293" t="n">
         <v>292</v>
       </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
       <c r="R293" t="inlineStr">
         <is>
           <t>FOX Noemie</t>
@@ -18191,6 +18386,11 @@
       <c r="K294" t="n">
         <v>293</v>
       </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="R294" t="inlineStr">
         <is>
           <t>PRIGENT Camille</t>
@@ -18254,6 +18454,11 @@
       <c r="K295" t="n">
         <v>294</v>
       </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="R295" t="inlineStr">
         <is>
           <t>HUG Angele</t>
@@ -18317,6 +18522,11 @@
       <c r="K296" t="n">
         <v>295</v>
       </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="R296" t="inlineStr">
         <is>
           <t>WOODS Kimberley</t>
@@ -18380,6 +18590,11 @@
       <c r="K297" t="n">
         <v>296</v>
       </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="R297" t="inlineStr">
         <is>
           <t>KITAMURA Koki</t>
@@ -18506,6 +18721,11 @@
       <c r="K299" t="n">
         <v>298</v>
       </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
       <c r="R299" t="inlineStr">
         <is>
           <t>NESHIME Daisuke</t>
@@ -18569,6 +18789,11 @@
       <c r="K300" t="n">
         <v>299</v>
       </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
       <c r="R300" t="inlineStr">
         <is>
           <t>MISHIMA Yu</t>
@@ -18632,6 +18857,11 @@
       <c r="K301" t="n">
         <v>300</v>
       </c>
+      <c r="M301" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
       <c r="R301" t="inlineStr">
         <is>
           <t>WILHELMER Noah</t>
@@ -18695,6 +18925,11 @@
       <c r="K302" t="n">
         <v>301</v>
       </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
       <c r="R302" t="inlineStr">
         <is>
           <t>SKUBIK David</t>
@@ -18821,6 +19056,11 @@
       <c r="K304" t="n">
         <v>303</v>
       </c>
+      <c r="M304" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
       <c r="R304" t="inlineStr">
         <is>
           <t>KRACHKO Arkhyp</t>
@@ -18884,6 +19124,11 @@
       <c r="K305" t="n">
         <v>304</v>
       </c>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="R305" t="inlineStr">
         <is>
           <t>BARAT Andy</t>
@@ -18947,6 +19192,11 @@
       <c r="K306" t="n">
         <v>305</v>
       </c>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
       <c r="R306" t="inlineStr">
         <is>
           <t>DA SILVA Kaua</t>
@@ -19010,6 +19260,11 @@
       <c r="K307" t="n">
         <v>306</v>
       </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
       <c r="R307" t="inlineStr">
         <is>
           <t>ANDERSON Finn</t>
@@ -19073,6 +19328,11 @@
       <c r="K308" t="n">
         <v>307</v>
       </c>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="R308" t="inlineStr">
         <is>
           <t>UKALOVIC Thomas</t>
@@ -19136,6 +19396,11 @@
       <c r="K309" t="n">
         <v>308</v>
       </c>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="R309" t="inlineStr">
         <is>
           <t>BOYD Trevor</t>
@@ -19199,6 +19464,11 @@
       <c r="K310" t="n">
         <v>309</v>
       </c>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="R310" t="inlineStr">
         <is>
           <t>CUNHA Joao</t>
@@ -19262,6 +19532,11 @@
       <c r="K311" t="n">
         <v>310</v>
       </c>
+      <c r="M311" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
       <c r="R311" t="inlineStr">
         <is>
           <t>BRZEZINSKI Jakub</t>
@@ -19325,6 +19600,11 @@
       <c r="K312" t="n">
         <v>311</v>
       </c>
+      <c r="M312" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="R312" t="inlineStr">
         <is>
           <t>LOCNIKAR Jan</t>
@@ -19388,6 +19668,11 @@
       <c r="K313" t="n">
         <v>312</v>
       </c>
+      <c r="M313" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
       <c r="R313" t="inlineStr">
         <is>
           <t>SOVKO Serhii</t>
@@ -19451,6 +19736,11 @@
       <c r="K314" t="n">
         <v>313</v>
       </c>
+      <c r="M314" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="R314" t="inlineStr">
         <is>
           <t>FRIEDENSON Kaelin</t>
@@ -19514,6 +19804,11 @@
       <c r="K315" t="n">
         <v>314</v>
       </c>
+      <c r="M315" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
       <c r="R315" t="inlineStr">
         <is>
           <t>RUDORFER Martin</t>
@@ -19577,6 +19872,11 @@
       <c r="K316" t="n">
         <v>315</v>
       </c>
+      <c r="M316" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="R316" t="inlineStr">
         <is>
           <t>FERRAZZI Xabier</t>
@@ -19640,6 +19940,11 @@
       <c r="K317" t="n">
         <v>316</v>
       </c>
+      <c r="M317" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="R317" t="inlineStr">
         <is>
           <t>LEITNER Mario</t>
@@ -19703,6 +20008,11 @@
       <c r="K318" t="n">
         <v>317</v>
       </c>
+      <c r="M318" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="R318" t="inlineStr">
         <is>
           <t>GRIGAR Jakub</t>
@@ -19766,6 +20076,11 @@
       <c r="K319" t="n">
         <v>318</v>
       </c>
+      <c r="M319" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="R319" t="inlineStr">
         <is>
           <t>MCCREERY Alistair</t>
@@ -19829,6 +20144,11 @@
       <c r="K320" t="n">
         <v>319</v>
       </c>
+      <c r="M320" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
       <c r="R320" t="inlineStr">
         <is>
           <t>ECHANIZ Pau</t>
@@ -19892,6 +20212,11 @@
       <c r="K321" t="n">
         <v>320</v>
       </c>
+      <c r="M321" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="R321" t="inlineStr">
         <is>
           <t>HALCIN Martin</t>
@@ -19955,6 +20280,11 @@
       <c r="K322" t="n">
         <v>321</v>
       </c>
+      <c r="M322" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="R322" t="inlineStr">
         <is>
           <t>OHRSTROM Isak</t>
@@ -20018,6 +20348,11 @@
       <c r="K323" t="n">
         <v>322</v>
       </c>
+      <c r="M323" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="R323" t="inlineStr">
         <is>
           <t>CURTIN Dominic</t>
@@ -20081,6 +20416,11 @@
       <c r="K324" t="n">
         <v>323</v>
       </c>
+      <c r="M324" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
       <c r="R324" t="inlineStr">
         <is>
           <t>ALVARENGA Frederico</t>
@@ -20144,6 +20484,11 @@
       <c r="K325" t="n">
         <v>324</v>
       </c>
+      <c r="M325" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="R325" t="inlineStr">
         <is>
           <t>IVCHENKO Artem</t>
@@ -20207,6 +20552,11 @@
       <c r="K326" t="n">
         <v>325</v>
       </c>
+      <c r="M326" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
       <c r="R326" t="inlineStr">
         <is>
           <t>SAVLI Jakob</t>
@@ -20270,6 +20620,11 @@
       <c r="K327" t="n">
         <v>326</v>
       </c>
+      <c r="M327" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="R327" t="inlineStr">
         <is>
           <t>COLLIER Nicholas</t>
@@ -20333,6 +20688,11 @@
       <c r="K328" t="n">
         <v>327</v>
       </c>
+      <c r="M328" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="R328" t="inlineStr">
         <is>
           <t>POPE Benjamin</t>
@@ -20396,6 +20756,11 @@
       <c r="K329" t="n">
         <v>328</v>
       </c>
+      <c r="M329" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
       <c r="R329" t="inlineStr">
         <is>
           <t>DESNOS Mathieu</t>
@@ -20459,6 +20824,11 @@
       <c r="K330" t="n">
         <v>329</v>
       </c>
+      <c r="M330" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="R330" t="inlineStr">
         <is>
           <t>LONG Kyler James</t>
@@ -20522,6 +20892,11 @@
       <c r="K331" t="n">
         <v>330</v>
       </c>
+      <c r="M331" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="R331" t="inlineStr">
         <is>
           <t>CASTRYCK Titouan</t>
@@ -20585,6 +20960,11 @@
       <c r="K332" t="n">
         <v>331</v>
       </c>
+      <c r="M332" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="R332" t="inlineStr">
         <is>
           <t>ROELLER Tillmann</t>
@@ -20648,6 +21028,11 @@
       <c r="K333" t="n">
         <v>332</v>
       </c>
+      <c r="M333" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="R333" t="inlineStr">
         <is>
           <t>NOVAK Matyas</t>
@@ -20711,6 +21096,11 @@
       <c r="K334" t="n">
         <v>333</v>
       </c>
+      <c r="M334" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="R334" t="inlineStr">
         <is>
           <t>HENGST Stefan</t>
@@ -20774,6 +21164,11 @@
       <c r="K335" t="n">
         <v>334</v>
       </c>
+      <c r="M335" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="R335" t="inlineStr">
         <is>
           <t>BALDONI Alex</t>
@@ -20837,6 +21232,11 @@
       <c r="K336" t="n">
         <v>335</v>
       </c>
+      <c r="M336" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="R336" t="inlineStr">
         <is>
           <t>LONG Merle</t>
@@ -20900,6 +21300,11 @@
       <c r="K337" t="n">
         <v>336</v>
       </c>
+      <c r="M337" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R337" t="inlineStr">
         <is>
           <t>KREJCI Jakub</t>
@@ -20963,6 +21368,11 @@
       <c r="K338" t="n">
         <v>337</v>
       </c>
+      <c r="M338" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="R338" t="inlineStr">
         <is>
           <t>CHIARELLO Gelindo</t>
@@ -21026,6 +21436,11 @@
       <c r="K339" t="n">
         <v>338</v>
       </c>
+      <c r="M339" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="R339" t="inlineStr">
         <is>
           <t>HOCEVAR Ziga Lin</t>
@@ -21089,6 +21504,11 @@
       <c r="K340" t="n">
         <v>339</v>
       </c>
+      <c r="M340" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="R340" t="inlineStr">
         <is>
           <t>QUAN Xin</t>
@@ -21152,6 +21572,11 @@
       <c r="K341" t="n">
         <v>340</v>
       </c>
+      <c r="M341" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="R341" t="inlineStr">
         <is>
           <t>LEAVER Sam</t>
@@ -21215,6 +21640,11 @@
       <c r="K342" t="n">
         <v>341</v>
       </c>
+      <c r="M342" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="R342" t="inlineStr">
         <is>
           <t>OSCHMAUTZ Felix</t>
@@ -21278,6 +21708,11 @@
       <c r="K343" t="n">
         <v>342</v>
       </c>
+      <c r="M343" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="R343" t="inlineStr">
         <is>
           <t>ROHRER Jan</t>
@@ -21341,6 +21776,11 @@
       <c r="K344" t="n">
         <v>343</v>
       </c>
+      <c r="M344" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
       <c r="R344" t="inlineStr">
         <is>
           <t>MADORE Mathurin</t>
@@ -21404,6 +21844,11 @@
       <c r="K345" t="n">
         <v>344</v>
       </c>
+      <c r="M345" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="R345" t="inlineStr">
         <is>
           <t>GONCALVES Pedro</t>
@@ -21467,6 +21912,11 @@
       <c r="K346" t="n">
         <v>345</v>
       </c>
+      <c r="M346" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="R346" t="inlineStr">
         <is>
           <t>HEGGE Noah</t>
@@ -21530,6 +21980,11 @@
       <c r="K347" t="n">
         <v>346</v>
       </c>
+      <c r="M347" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="R347" t="inlineStr">
         <is>
           <t>DICKSON Jonny</t>
@@ -21593,6 +22048,11 @@
       <c r="K348" t="n">
         <v>347</v>
       </c>
+      <c r="M348" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="R348" t="inlineStr">
         <is>
           <t>RENIA Benjamin</t>
@@ -21656,6 +22116,11 @@
       <c r="K349" t="n">
         <v>348</v>
       </c>
+      <c r="M349" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="R349" t="inlineStr">
         <is>
           <t>POLACZYK Mateusz</t>
@@ -21719,6 +22184,11 @@
       <c r="K350" t="n">
         <v>349</v>
       </c>
+      <c r="M350" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="R350" t="inlineStr">
         <is>
           <t>OCHOA Manuel</t>
@@ -21782,6 +22252,11 @@
       <c r="K351" t="n">
         <v>350</v>
       </c>
+      <c r="M351" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="R351" t="inlineStr">
         <is>
           <t>LLORENTE David</t>
@@ -21845,6 +22320,11 @@
       <c r="K352" t="n">
         <v>351</v>
       </c>
+      <c r="M352" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="R352" t="inlineStr">
         <is>
           <t>DOUGOUD Martin</t>
@@ -21907,6 +22387,11 @@
       </c>
       <c r="K353" t="n">
         <v>352</v>
+      </c>
+      <c r="M353" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="R353" t="inlineStr">
         <is>

</xml_diff>